<commit_message>
Exclude irretrievable PDFs from screening2 analysis
- Add pdf_irretrievable filter in process_review_repredicting() for
  screening2 to ensure only records with accessible PDFs are analyzed
- Regenerate all performance metrics, tables, and plots with corrected data
- Add paper.md to .gitignore

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/validation/results/results/Supplementary_Table_S3_Performance_Metrics.xlsx
+++ b/validation/results/results/Supplementary_Table_S3_Performance_Metrics.xlsx
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>167</v>
@@ -812,10 +812,10 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>5566</v>
+        <v>4366</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>5566</v>
+        <v>4366</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>0</v>
@@ -824,46 +824,46 @@
         <v>133</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>5288</v>
+        <v>4097</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>95</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>0.727</v>
+        <v>0.764</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>0.583</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>0.647</v>
+        <v>0.662</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0.638</v>
+        <v>0.652</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0.634</v>
+        <v>0.646</v>
       </c>
       <c r="Q4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>0.727</v>
+        <v>0.764</v>
       </c>
       <c r="S4" s="3" t="n">
         <v>0.583</v>
       </c>
       <c r="T4" s="3" t="n">
-        <v>0.647</v>
+        <v>0.662</v>
       </c>
       <c r="U4" s="3" t="n">
-        <v>0.638</v>
+        <v>0.652</v>
       </c>
       <c r="V4" s="3" t="n">
-        <v>0.634</v>
+        <v>0.646</v>
       </c>
     </row>
     <row r="5">
@@ -888,13 +888,13 @@
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>228</v>
+        <v>210</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" s="5" t="n">
         <v>131</v>
@@ -903,43 +903,43 @@
         <v>38</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="K5" s="5" t="n">
         <v>17</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>0.819</v>
+        <v>0.845</v>
       </c>
       <c r="M5" s="5" t="n">
         <v>0.885</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>0.851</v>
+        <v>0.865</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>0.48</v>
+        <v>0.517</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>0.476</v>
+        <v>0.515</v>
       </c>
       <c r="Q5" s="5" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.995</v>
       </c>
       <c r="R5" s="5" t="n">
-        <v>0.772</v>
+        <v>0.841</v>
       </c>
       <c r="S5" s="5" t="n">
-        <v>0.835</v>
+        <v>0.881</v>
       </c>
       <c r="T5" s="5" t="n">
-        <v>0.802</v>
+        <v>0.861</v>
       </c>
       <c r="U5" s="5" t="n">
-        <v>0.453</v>
+        <v>0.514</v>
       </c>
       <c r="V5" s="5" t="n">
-        <v>0.448</v>
+        <v>0.512</v>
       </c>
     </row>
     <row r="6">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>167</v>
@@ -1116,10 +1116,10 @@
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>5566</v>
+        <v>4366</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>5566</v>
+        <v>4366</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>0</v>
@@ -1128,46 +1128,46 @@
         <v>158</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>5276</v>
+        <v>4086</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="K8" s="3" t="n">
         <v>70</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>0.718</v>
+        <v>0.752</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>0.6929999999999999</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>0.705</v>
+        <v>0.721</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0.6929999999999999</v>
+        <v>0.707</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>0.6929999999999999</v>
+        <v>0.707</v>
       </c>
       <c r="Q8" s="3" t="n">
         <v>1</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>0.718</v>
+        <v>0.752</v>
       </c>
       <c r="S8" s="3" t="n">
         <v>0.6929999999999999</v>
       </c>
       <c r="T8" s="3" t="n">
-        <v>0.705</v>
+        <v>0.721</v>
       </c>
       <c r="U8" s="3" t="n">
-        <v>0.6929999999999999</v>
+        <v>0.707</v>
       </c>
       <c r="V8" s="3" t="n">
-        <v>0.6929999999999999</v>
+        <v>0.707</v>
       </c>
     </row>
     <row r="9">
@@ -1192,13 +1192,13 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>228</v>
+        <v>210</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" s="5" t="n">
         <v>132</v>
@@ -1207,43 +1207,43 @@
         <v>35</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="K9" s="5" t="n">
         <v>16</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>0.805</v>
+        <v>0.83</v>
       </c>
       <c r="M9" s="5" t="n">
         <v>0.892</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>0.846</v>
+        <v>0.86</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>0.451</v>
+        <v>0.486</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>0.443</v>
+        <v>0.481</v>
       </c>
       <c r="Q9" s="5" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.995</v>
       </c>
       <c r="R9" s="5" t="n">
-        <v>0.759</v>
+        <v>0.826</v>
       </c>
       <c r="S9" s="5" t="n">
-        <v>0.841</v>
+        <v>0.888</v>
       </c>
       <c r="T9" s="5" t="n">
-        <v>0.798</v>
+        <v>0.856</v>
       </c>
       <c r="U9" s="5" t="n">
-        <v>0.425</v>
+        <v>0.483</v>
       </c>
       <c r="V9" s="5" t="n">
-        <v>0.418</v>
+        <v>0.479</v>
       </c>
     </row>
     <row r="10">
@@ -1344,7 +1344,7 @@
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>167</v>
@@ -1420,10 +1420,10 @@
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>5566</v>
+        <v>4366</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>5566</v>
+        <v>4366</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>0</v>
@@ -1432,46 +1432,46 @@
         <v>162</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>5246</v>
+        <v>4062</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="K12" s="3" t="n">
         <v>66</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0.638</v>
+        <v>0.681</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0.711</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.672</v>
+        <v>0.695</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>0.658</v>
+        <v>0.678</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>0.657</v>
+        <v>0.678</v>
       </c>
       <c r="Q12" s="3" t="n">
         <v>1</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>0.638</v>
+        <v>0.681</v>
       </c>
       <c r="S12" s="3" t="n">
         <v>0.711</v>
       </c>
       <c r="T12" s="3" t="n">
-        <v>0.672</v>
+        <v>0.695</v>
       </c>
       <c r="U12" s="3" t="n">
-        <v>0.658</v>
+        <v>0.678</v>
       </c>
       <c r="V12" s="3" t="n">
-        <v>0.657</v>
+        <v>0.678</v>
       </c>
     </row>
     <row r="13">
@@ -1496,13 +1496,13 @@
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>228</v>
+        <v>209</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H13" s="5" t="n">
         <v>131</v>
@@ -1511,43 +1511,43 @@
         <v>34</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="K13" s="5" t="n">
         <v>17</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>0.804</v>
+        <v>0.829</v>
       </c>
       <c r="M13" s="5" t="n">
         <v>0.885</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>0.842</v>
+        <v>0.856</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>0.434</v>
+        <v>0.468</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>0.427</v>
+        <v>0.465</v>
       </c>
       <c r="Q13" s="5" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.991</v>
       </c>
       <c r="R13" s="5" t="n">
-        <v>0.754</v>
+        <v>0.821</v>
       </c>
       <c r="S13" s="5" t="n">
-        <v>0.831</v>
+        <v>0.877</v>
       </c>
       <c r="T13" s="5" t="n">
-        <v>0.791</v>
+        <v>0.848</v>
       </c>
       <c r="U13" s="5" t="n">
-        <v>0.407</v>
+        <v>0.464</v>
       </c>
       <c r="V13" s="5" t="n">
-        <v>0.401</v>
+        <v>0.461</v>
       </c>
     </row>
     <row r="14">
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>4501</v>
+        <v>4497</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>4497</v>
@@ -1648,7 +1648,7 @@
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>167</v>
@@ -1724,10 +1724,10 @@
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>5566</v>
+        <v>4366</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>5566</v>
+        <v>4366</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>0</v>
@@ -1736,46 +1736,46 @@
         <v>111</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>5293</v>
+        <v>4098</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="K16" s="3" t="n">
         <v>117</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>0.712</v>
+        <v>0.735</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>0.487</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.578</v>
+        <v>0.586</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.575</v>
+        <v>0.581</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="Q16" s="3" t="n">
         <v>1</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>0.712</v>
+        <v>0.735</v>
       </c>
       <c r="S16" s="3" t="n">
         <v>0.487</v>
       </c>
       <c r="T16" s="3" t="n">
-        <v>0.578</v>
+        <v>0.586</v>
       </c>
       <c r="U16" s="3" t="n">
-        <v>0.575</v>
+        <v>0.581</v>
       </c>
       <c r="V16" s="3" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.5679999999999999</v>
       </c>
     </row>
     <row r="17">
@@ -1800,58 +1800,58 @@
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>228</v>
+        <v>209</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H17" s="5" t="n">
         <v>78</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="K17" s="5" t="n">
         <v>69</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>0.736</v>
+        <v>0.765</v>
       </c>
       <c r="M17" s="5" t="n">
         <v>0.531</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>0.617</v>
+        <v>0.627</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>0.105</v>
+        <v>0.131</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>0.097</v>
+        <v>0.119</v>
       </c>
       <c r="Q17" s="5" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.991</v>
       </c>
       <c r="R17" s="5" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.757</v>
       </c>
       <c r="S17" s="5" t="n">
-        <v>0.498</v>
+        <v>0.526</v>
       </c>
       <c r="T17" s="5" t="n">
-        <v>0.579</v>
+        <v>0.621</v>
       </c>
       <c r="U17" s="5" t="n">
-        <v>0.098</v>
+        <v>0.13</v>
       </c>
       <c r="V17" s="5" t="n">
-        <v>0.091</v>
+        <v>0.117</v>
       </c>
     </row>
     <row r="18">
@@ -1952,7 +1952,7 @@
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>167</v>
@@ -2028,10 +2028,10 @@
         </is>
       </c>
       <c r="E20" s="3" t="n">
-        <v>5566</v>
+        <v>4366</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>5566</v>
+        <v>4366</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>0</v>
@@ -2040,46 +2040,46 @@
         <v>156</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>5300</v>
+        <v>4107</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="K20" s="3" t="n">
         <v>72</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>0.804</v>
+        <v>0.834</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>0.6840000000000001</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>0.739</v>
+        <v>0.752</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>0.732</v>
+        <v>0.744</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>0.729</v>
+        <v>0.74</v>
       </c>
       <c r="Q20" s="3" t="n">
         <v>1</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>0.804</v>
+        <v>0.834</v>
       </c>
       <c r="S20" s="3" t="n">
         <v>0.6840000000000001</v>
       </c>
       <c r="T20" s="3" t="n">
-        <v>0.739</v>
+        <v>0.752</v>
       </c>
       <c r="U20" s="3" t="n">
-        <v>0.732</v>
+        <v>0.744</v>
       </c>
       <c r="V20" s="3" t="n">
-        <v>0.729</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="21">
@@ -2104,13 +2104,13 @@
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>228</v>
+        <v>210</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H21" s="5" t="n">
         <v>126</v>
@@ -2119,43 +2119,43 @@
         <v>38</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="K21" s="5" t="n">
         <v>22</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.84</v>
       </c>
       <c r="M21" s="5" t="n">
         <v>0.851</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>0.832</v>
+        <v>0.846</v>
       </c>
       <c r="O21" s="5" t="n">
-        <v>0.432</v>
+        <v>0.469</v>
       </c>
       <c r="P21" s="5" t="n">
-        <v>0.431</v>
+        <v>0.469</v>
       </c>
       <c r="Q21" s="5" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.995</v>
       </c>
       <c r="R21" s="5" t="n">
-        <v>0.767</v>
+        <v>0.836</v>
       </c>
       <c r="S21" s="5" t="n">
-        <v>0.803</v>
+        <v>0.847</v>
       </c>
       <c r="T21" s="5" t="n">
-        <v>0.784</v>
+        <v>0.842</v>
       </c>
       <c r="U21" s="5" t="n">
-        <v>0.408</v>
+        <v>0.467</v>
       </c>
       <c r="V21" s="5" t="n">
-        <v>0.406</v>
+        <v>0.466</v>
       </c>
     </row>
     <row r="22">
@@ -2256,7 +2256,7 @@
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>167</v>
@@ -2332,10 +2332,10 @@
         </is>
       </c>
       <c r="E24" s="3" t="n">
-        <v>5566</v>
+        <v>4366</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>5566</v>
+        <v>4366</v>
       </c>
       <c r="G24" s="3" t="n">
         <v>0</v>
@@ -2344,46 +2344,46 @@
         <v>147</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>5272</v>
+        <v>4079</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="K24" s="3" t="n">
         <v>81</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.714</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>0.645</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>0.667</v>
+        <v>0.677</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>0.653</v>
+        <v>0.662</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>0.653</v>
+        <v>0.661</v>
       </c>
       <c r="Q24" s="3" t="n">
         <v>1</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.714</v>
       </c>
       <c r="S24" s="3" t="n">
         <v>0.645</v>
       </c>
       <c r="T24" s="3" t="n">
-        <v>0.667</v>
+        <v>0.677</v>
       </c>
       <c r="U24" s="3" t="n">
-        <v>0.653</v>
+        <v>0.662</v>
       </c>
       <c r="V24" s="3" t="n">
-        <v>0.653</v>
+        <v>0.661</v>
       </c>
     </row>
     <row r="25">
@@ -2408,13 +2408,13 @@
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>228</v>
+        <v>210</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H25" s="5" t="n">
         <v>122</v>
@@ -2423,43 +2423,43 @@
         <v>37</v>
       </c>
       <c r="J25" s="5" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="K25" s="5" t="n">
         <v>26</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>0.803</v>
+        <v>0.83</v>
       </c>
       <c r="M25" s="5" t="n">
         <v>0.824</v>
       </c>
       <c r="N25" s="5" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.827</v>
       </c>
       <c r="O25" s="5" t="n">
-        <v>0.383</v>
+        <v>0.419</v>
       </c>
       <c r="P25" s="5" t="n">
-        <v>0.383</v>
+        <v>0.419</v>
       </c>
       <c r="Q25" s="5" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.995</v>
       </c>
       <c r="R25" s="5" t="n">
-        <v>0.757</v>
+        <v>0.826</v>
       </c>
       <c r="S25" s="5" t="n">
-        <v>0.777</v>
+        <v>0.82</v>
       </c>
       <c r="T25" s="5" t="n">
-        <v>0.767</v>
+        <v>0.823</v>
       </c>
       <c r="U25" s="5" t="n">
-        <v>0.361</v>
+        <v>0.417</v>
       </c>
       <c r="V25" s="5" t="n">
-        <v>0.361</v>
+        <v>0.417</v>
       </c>
     </row>
   </sheetData>
@@ -2553,34 +2553,34 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>0.605</v>
+        <v>0.621</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>0.699</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.637</v>
+        <v>0.644</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.463</v>
+        <v>0.475</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.452</v>
+        <v>0.465</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>0.589</v>
+        <v>0.616</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.68</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.62</v>
+        <v>0.638</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.453</v>
+        <v>0.472</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>0.443</v>
+        <v>0.462</v>
       </c>
     </row>
     <row r="3">
@@ -2590,34 +2590,34 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>0.611</v>
+        <v>0.626</v>
       </c>
       <c r="C3" s="5" t="n">
         <v>0.652</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>0.63</v>
+        <v>0.638</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.449</v>
+        <v>0.461</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.447</v>
+        <v>0.46</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>0.596</v>
+        <v>0.621</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>0.635</v>
+        <v>0.647</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>0.614</v>
+        <v>0.632</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>0.441</v>
+        <v>0.459</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>0.438</v>
+        <v>0.457</v>
       </c>
     </row>
     <row r="4">
@@ -2627,34 +2627,34 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>0.661</v>
+        <v>0.676</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>0.526</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.575</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.404</v>
+        <v>0.417</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.393</v>
+        <v>0.405</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.645</v>
+        <v>0.67</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.511</v>
+        <v>0.522</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.553</v>
+        <v>0.57</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.397</v>
+        <v>0.414</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.385</v>
+        <v>0.403</v>
       </c>
     </row>
     <row r="5">
@@ -2664,34 +2664,34 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.541</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>0.6830000000000001</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0.596</v>
+        <v>0.605</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.396</v>
+        <v>0.409</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.386</v>
+        <v>0.401</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.525</v>
+        <v>0.552</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>0.665</v>
+        <v>0.676</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>0.579</v>
+        <v>0.599</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>0.387</v>
+        <v>0.407</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>0.378</v>
+        <v>0.398</v>
       </c>
     </row>
     <row r="6">
@@ -2701,34 +2701,34 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0.659</v>
+        <v>0.672</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>0.485</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.531</v>
+        <v>0.538</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.379</v>
+        <v>0.39</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.36</v>
+        <v>0.371</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.643</v>
+        <v>0.666</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.47</v>
+        <v>0.481</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.517</v>
+        <v>0.533</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.371</v>
+        <v>0.387</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0.353</v>
+        <v>0.369</v>
       </c>
     </row>
     <row r="7">
@@ -2738,34 +2738,34 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>0.516</v>
+        <v>0.53</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>0.386</v>
       </c>
       <c r="D7" s="5" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0.231</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.223</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0.524</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>0.383</v>
+      </c>
+      <c r="I7" s="5" t="n">
         <v>0.436</v>
       </c>
-      <c r="E7" s="5" t="n">
-        <v>0.223</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>0.216</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>0.502</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>0.376</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>0.424</v>
-      </c>
       <c r="J7" s="5" t="n">
-        <v>0.221</v>
+        <v>0.23</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>0.214</v>
+        <v>0.222</v>
       </c>
     </row>
   </sheetData>
@@ -2870,34 +2870,34 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.518</v>
+        <v>0.537</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>0.571</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.523</v>
+        <v>0.53</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0.512</v>
+        <v>0.519</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>0.501</v>
+        <v>0.506</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.518</v>
+        <v>0.537</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0.571</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.523</v>
+        <v>0.53</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>0.512</v>
+        <v>0.519</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v>0.501</v>
+        <v>0.506</v>
       </c>
     </row>
     <row r="3">
@@ -2912,34 +2912,34 @@
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>0.526</v>
+        <v>0.543</v>
       </c>
       <c r="D3" s="5" t="n">
         <v>0.547</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.535</v>
+        <v>0.543</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.516</v>
+        <v>0.523</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>0.515</v>
+        <v>0.522</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>0.526</v>
+        <v>0.543</v>
       </c>
       <c r="I3" s="5" t="n">
         <v>0.547</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>0.535</v>
+        <v>0.543</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>0.516</v>
+        <v>0.523</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>0.515</v>
+        <v>0.522</v>
       </c>
     </row>
     <row r="4">
@@ -2954,34 +2954,34 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.424</v>
+        <v>0.446</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>0.591</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.482</v>
+        <v>0.493</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.467</v>
+        <v>0.477</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.455</v>
+        <v>0.465</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.424</v>
+        <v>0.446</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0.591</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>0.482</v>
+        <v>0.493</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0.467</v>
+        <v>0.477</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>0.455</v>
+        <v>0.465</v>
       </c>
     </row>
     <row r="5">
@@ -2996,34 +2996,34 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>0.426</v>
+        <v>0.438</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>0.348</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.373</v>
+        <v>0.377</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.353</v>
+        <v>0.356</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.346</v>
+        <v>0.348</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>0.426</v>
+        <v>0.438</v>
       </c>
       <c r="I5" s="5" t="n">
         <v>0.348</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>0.373</v>
+        <v>0.377</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>0.353</v>
+        <v>0.356</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>0.346</v>
+        <v>0.348</v>
       </c>
     </row>
     <row r="6">
@@ -3038,34 +3038,34 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.628</v>
+        <v>0.643</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>0.409</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.473</v>
+        <v>0.479</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.481</v>
+        <v>0.487</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.461</v>
+        <v>0.466</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.628</v>
+        <v>0.643</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>0.409</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0.473</v>
+        <v>0.479</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0.481</v>
+        <v>0.487</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>0.461</v>
+        <v>0.466</v>
       </c>
     </row>
     <row r="7">
@@ -3080,34 +3080,34 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>0.601</v>
+        <v>0.613</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>0.383</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.432</v>
+        <v>0.437</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.445</v>
+        <v>0.449</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0.419</v>
+        <v>0.423</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>0.601</v>
+        <v>0.613</v>
       </c>
       <c r="I7" s="5" t="n">
         <v>0.383</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.432</v>
+        <v>0.437</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>0.445</v>
+        <v>0.449</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>0.419</v>
+        <v>0.423</v>
       </c>
     </row>
     <row r="8">
@@ -3122,34 +3122,34 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.704</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>0.827</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.75</v>
+        <v>0.757</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.414</v>
+        <v>0.432</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0.404</v>
+        <v>0.423</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.66</v>
+        <v>0.694</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>0.79</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.717</v>
+        <v>0.746</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>0.395</v>
+        <v>0.426</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>0.385</v>
+        <v>0.417</v>
       </c>
     </row>
     <row r="9">
@@ -3164,34 +3164,34 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>0.697</v>
+        <v>0.71</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>0.758</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.726</v>
+        <v>0.733</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.383</v>
+        <v>0.4</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0.379</v>
+        <v>0.398</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>0.665</v>
+        <v>0.699</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>0.723</v>
+        <v>0.746</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>0.6929999999999999</v>
+        <v>0.722</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>0.365</v>
+        <v>0.394</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>0.362</v>
+        <v>0.392</v>
       </c>
     </row>
     <row r="10">
@@ -3206,34 +3206,34 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.657</v>
+        <v>0.67</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>0.776</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.711</v>
+        <v>0.717</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.324</v>
+        <v>0.342</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0.318</v>
+        <v>0.337</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.625</v>
+        <v>0.659</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.739</v>
+        <v>0.762</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>0.676</v>
+        <v>0.705</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0.308</v>
+        <v>0.336</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0.302</v>
+        <v>0.331</v>
       </c>
     </row>
     <row r="11">
@@ -3248,34 +3248,34 @@
         </is>
       </c>
       <c r="C11" s="5" t="n">
-        <v>0.607</v>
+        <v>0.621</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>0.425</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.5</v>
+        <v>0.505</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.093</v>
+        <v>0.106</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.098</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>0.578</v>
+        <v>0.611</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.404</v>
+        <v>0.418</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.475</v>
+        <v>0.496</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>0.089</v>
+        <v>0.105</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>0.083</v>
+        <v>0.097</v>
       </c>
     </row>
     <row r="12">
@@ -3290,34 +3290,34 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.695</v>
+        <v>0.708</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>0.643</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.664</v>
+        <v>0.671</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.328</v>
+        <v>0.346</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.325</v>
+        <v>0.343</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.663</v>
+        <v>0.698</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.612</v>
+        <v>0.635</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>0.633</v>
+        <v>0.662</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0.312</v>
+        <v>0.342</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0.309</v>
+        <v>0.339</v>
       </c>
     </row>
     <row r="13">
@@ -3332,34 +3332,34 @@
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>0.717</v>
+        <v>0.731</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>0.586</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.631</v>
+        <v>0.638</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.312</v>
+        <v>0.33</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.301</v>
+        <v>0.319</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.72</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.579</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.601</v>
+        <v>0.629</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>0.298</v>
+        <v>0.325</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>0.287</v>
+        <v>0.315</v>
       </c>
     </row>
   </sheetData>

</xml_diff>